<commit_message>
Restore the café hero background image
The hero-media parser only matched images inside a media wrapper or as a
direct child, and left relative image sources un-absolutized, so the
café hero's plain <img> background was dropped and the block fell back
to its image-less dark variant. Absolutize image URLs and fall back to
the first non-icon image in the section, restoring the full-bleed café
interior background with its cream headline and amber eyebrow.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-cafe.report.xlsx
+++ b/tools/importer/reports/import-cafe.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="66">
   <si>
     <t>_reportFile</t>
   </si>
@@ -37,6 +37,51 @@
     <t>url</t>
   </si>
   <si>
+    <t>frescopa-atelier/article.report.json</t>
+  </si>
+  <si>
+    <t>["article-body"]</t>
+  </si>
+  <si>
+    <t>frescopa-atelier/article</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>article</t>
+  </si>
+  <si>
+    <t>2026-07-17T13:09:24.195Z</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>https://markszulc.github.io/frescopa-atelier/article.html</t>
+  </si>
+  <si>
+    <t>frescopa-atelier/atelier.report.json</t>
+  </si>
+  <si>
+    <t>["product-hero","product-jumpnav","steps-tabs","media-video","accordion","accordion","spec-table","taste-profile","reviews","bundle-cards","cards-product"]</t>
+  </si>
+  <si>
+    <t>frescopa-atelier/atelier</t>
+  </si>
+  <si>
+    <t>atelier</t>
+  </si>
+  <si>
+    <t>2026-07-18T08:12:40.058Z</t>
+  </si>
+  <si>
+    <t>The Atelier — Fréscopa</t>
+  </si>
+  <si>
+    <t>https://markszulc.github.io/frescopa-atelier/atelier.html</t>
+  </si>
+  <si>
     <t>frescopa-atelier/beverages.report.json</t>
   </si>
   <si>
@@ -46,16 +91,10 @@
     <t>frescopa-atelier/beverages</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
     <t>beverages</t>
   </si>
   <si>
-    <t>2026-07-15T23:25:45.892Z</t>
-  </si>
-  <si>
-    <t/>
+    <t>2026-07-15T23:45:17.273Z</t>
   </si>
   <si>
     <t>https://markszulc.github.io/frescopa-atelier/beverages.html</t>
@@ -91,12 +130,30 @@
     <t>cafe</t>
   </si>
   <si>
-    <t>2026-07-15T23:26:18.079Z</t>
+    <t>2026-07-18T08:44:49.841Z</t>
   </si>
   <si>
     <t>https://markszulc.github.io/frescopa-atelier/cafe.html</t>
   </si>
   <si>
+    <t>frescopa-atelier/coffee.report.json</t>
+  </si>
+  <si>
+    <t>["machine-filter","cards-coffee","cards-coffee","cards-coffee"]</t>
+  </si>
+  <si>
+    <t>frescopa-atelier/coffee</t>
+  </si>
+  <si>
+    <t>coffee</t>
+  </si>
+  <si>
+    <t>2026-07-17T12:36:13.251Z</t>
+  </si>
+  <si>
+    <t>https://markszulc.github.io/frescopa-atelier/coffee.html</t>
+  </si>
+  <si>
     <t>frescopa-atelier/index.report.json</t>
   </si>
   <si>
@@ -116,6 +173,42 @@
   </si>
   <si>
     <t>https://markszulc.github.io/frescopa-atelier/index.html</t>
+  </si>
+  <si>
+    <t>frescopa-atelier/machines.report.json</t>
+  </si>
+  <si>
+    <t>["machine-filter","cards-machine","cards-machine","cards-machine","cards-machine"]</t>
+  </si>
+  <si>
+    <t>frescopa-atelier/machines</t>
+  </si>
+  <si>
+    <t>machines</t>
+  </si>
+  <si>
+    <t>2026-07-17T12:05:35.729Z</t>
+  </si>
+  <si>
+    <t>https://markszulc.github.io/frescopa-atelier/machines.html</t>
+  </si>
+  <si>
+    <t>frescopa-atelier/myatelier.report.json</t>
+  </si>
+  <si>
+    <t>["account-signin"]</t>
+  </si>
+  <si>
+    <t>frescopa-atelier/myatelier</t>
+  </si>
+  <si>
+    <t>myatelier</t>
+  </si>
+  <si>
+    <t>2026-07-17T12:45:04.895Z</t>
+  </si>
+  <si>
+    <t>https://markszulc.github.io/frescopa-atelier/myatelier.html</t>
   </si>
 </sst>
 </file>
@@ -504,7 +597,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -588,62 +681,192 @@
         <v>20</v>
       </c>
       <c r="G3" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="H3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D4" t="s">
         <v>11</v>
       </c>
       <c r="E4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G4" t="s">
         <v>14</v>
       </c>
       <c r="H4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D5" t="s">
         <v>11</v>
       </c>
       <c r="E5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G5" t="s">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="H5" t="s">
         <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>38</v>
+      </c>
+      <c r="F6" t="s">
+        <v>39</v>
+      </c>
+      <c r="G6" t="s">
+        <v>14</v>
+      </c>
+      <c r="H6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>44</v>
+      </c>
+      <c r="F7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>50</v>
+      </c>
+      <c r="F8" t="s">
+        <v>51</v>
+      </c>
+      <c r="G8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>57</v>
+      </c>
+      <c r="F9" t="s">
+        <v>58</v>
+      </c>
+      <c r="G9" t="s">
+        <v>14</v>
+      </c>
+      <c r="H9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>60</v>
+      </c>
+      <c r="B10" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10" t="s">
+        <v>62</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>63</v>
+      </c>
+      <c r="F10" t="s">
+        <v>64</v>
+      </c>
+      <c r="G10" t="s">
+        <v>14</v>
+      </c>
+      <c r="H10" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Restore the cafe locations store-locator and stats section
The columns-editorial block mapped "#locations article", which matched
all 26 nested store-locator cafe cards (plus the flagship) and replaced
them before the store-locator parser ran — leaving the section with no
store-locator block and 30 stray columns-editorial blocks. Scope the
flagship to "#locations > div > article" so the store-locator keeps its
26 location cards and renders the sticky map, scrollable list, search
and region filters as in the original.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-cafe.report.xlsx
+++ b/tools/importer/reports/import-cafe.report.xlsx
@@ -121,7 +121,7 @@
     <t>frescopa-atelier/cafe.report.json</t>
   </si>
   <si>
-    <t>["hero-media","hero-media","cards-reasons","columns-editorial","columns-editorial","columns-editorial","columns-editorial","columns-editorial","columns-editorial","columns-editorial","columns-editorial","columns-editorial","columns-editorial","columns-editorial","columns-editorial","columns-editorial","columns-editorial","columns-editorial","columns-editorial","columns-editorial","columns-editorial","columns-editorial","columns-editorial","columns-editorial","columns-editorial","columns-editorial","columns-editorial","columns-editorial","columns-editorial","columns-editorial","columns-editorial","columns-editorial","columns-editorial","cards-event","stats-row","store-locator","booking-form"]</t>
+    <t>["hero-media","hero-media","cards-reasons","columns-editorial","columns-editorial","columns-editorial","columns-editorial","cards-event","stats-row","store-locator","booking-form"]</t>
   </si>
   <si>
     <t>frescopa-atelier/cafe</t>
@@ -130,7 +130,7 @@
     <t>cafe</t>
   </si>
   <si>
-    <t>2026-07-18T08:44:49.841Z</t>
+    <t>2026-07-18T08:58:46.934Z</t>
   </si>
   <si>
     <t>https://markszulc.github.io/frescopa-atelier/cafe.html</t>

</xml_diff>